<commit_message>
scra sep 9 26
</commit_message>
<xml_diff>
--- a/scra/scra_pymt_history_from_2021.xlsx
+++ b/scra/scra_pymt_history_from_2021.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$L$99</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -1386,7 +1386,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q117"/>
@@ -1440,7 +1440,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1481,7 +1481,7 @@
       <c r="P2" s="11"/>
       <c r="Q2" s="12"/>
     </row>
-    <row r="3" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <f t="shared" ref="A3:A34" si="0">A2+1</f>
         <v>2</v>
@@ -1525,7 +1525,7 @@
       <c r="P3" s="11"/>
       <c r="Q3" s="12"/>
     </row>
-    <row r="4" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -1568,7 +1568,7 @@
       <c r="O4" s="11"/>
       <c r="Q4" s="12"/>
     </row>
-    <row r="5" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1681,8 +1681,8 @@
       <c r="J7" s="8">
         <v>1500</v>
       </c>
-      <c r="K7" s="36">
-        <v>0</v>
+      <c r="K7" s="18">
+        <v>2500</v>
       </c>
       <c r="L7" s="49" t="s">
         <v>169</v>
@@ -1807,8 +1807,8 @@
       <c r="J10" s="9">
         <v>7500</v>
       </c>
-      <c r="K10" s="36">
-        <v>0</v>
+      <c r="K10" s="18">
+        <v>7500</v>
       </c>
       <c r="L10" s="9"/>
       <c r="M10" s="10"/>
@@ -1817,7 +1817,7 @@
       <c r="P10" s="11"/>
       <c r="Q10" s="12"/>
     </row>
-    <row r="11" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="47">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1859,7 +1859,7 @@
       <c r="P11" s="11"/>
       <c r="Q11" s="12"/>
     </row>
-    <row r="12" spans="1:17" s="13" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" s="13" customFormat="1" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1903,7 +1903,7 @@
       <c r="P12" s="11"/>
       <c r="Q12" s="12"/>
     </row>
-    <row r="13" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1991,7 +1991,7 @@
       <c r="P14" s="11"/>
       <c r="Q14" s="12"/>
     </row>
-    <row r="15" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="51">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2033,7 +2033,7 @@
       <c r="P15" s="11"/>
       <c r="Q15" s="12"/>
     </row>
-    <row r="16" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="51">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2261,7 +2261,7 @@
       <c r="P21" s="11"/>
       <c r="Q21" s="12"/>
     </row>
-    <row r="22" spans="1:17" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" s="13" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2379,8 +2379,8 @@
       <c r="J24" s="18">
         <v>7500</v>
       </c>
-      <c r="K24" s="36">
-        <v>0</v>
+      <c r="K24" s="18">
+        <v>7500</v>
       </c>
       <c r="L24" s="9"/>
       <c r="M24" s="10"/>
@@ -2389,7 +2389,7 @@
       <c r="P24" s="11"/>
       <c r="Q24" s="12"/>
     </row>
-    <row r="25" spans="1:17" s="13" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" s="13" customFormat="1" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -2515,7 +2515,7 @@
       <c r="P27" s="11"/>
       <c r="Q27" s="12"/>
     </row>
-    <row r="28" spans="1:17" s="13" customFormat="1" ht="32.25" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" s="13" customFormat="1" ht="32.25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
         <f t="shared" si="0"/>
         <v>27</v>
@@ -2683,7 +2683,7 @@
       <c r="P31" s="11"/>
       <c r="Q31" s="12"/>
     </row>
-    <row r="32" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
         <f t="shared" si="0"/>
         <v>31</v>
@@ -2809,7 +2809,7 @@
       <c r="P34" s="11"/>
       <c r="Q34" s="12"/>
     </row>
-    <row r="35" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
         <f t="shared" ref="A35:A66" si="1">A34+1</f>
         <v>34</v>
@@ -2893,7 +2893,7 @@
       <c r="P36" s="11"/>
       <c r="Q36" s="12"/>
     </row>
-    <row r="37" spans="1:17" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" s="13" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="51">
         <f t="shared" si="1"/>
         <v>36</v>
@@ -3091,7 +3091,7 @@
       <c r="P41" s="11"/>
       <c r="Q41" s="12"/>
     </row>
-    <row r="42" spans="1:17" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" s="13" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="55">
         <f t="shared" si="1"/>
         <v>41</v>
@@ -3241,8 +3241,8 @@
       <c r="J45" s="9">
         <v>7500</v>
       </c>
-      <c r="K45" s="36">
-        <v>0</v>
+      <c r="K45" s="18">
+        <v>2500</v>
       </c>
       <c r="L45" s="9" t="s">
         <v>196</v>
@@ -3589,7 +3589,7 @@
       <c r="P53" s="11"/>
       <c r="Q53" s="12"/>
     </row>
-    <row r="54" spans="1:17" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" s="13" customFormat="1" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="47">
         <f t="shared" si="1"/>
         <v>53</v>
@@ -3631,7 +3631,7 @@
       <c r="P54" s="11"/>
       <c r="Q54" s="12"/>
     </row>
-    <row r="55" spans="1:17" s="13" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" s="13" customFormat="1" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
         <f t="shared" si="1"/>
         <v>54</v>
@@ -3719,7 +3719,7 @@
       <c r="P56" s="11"/>
       <c r="Q56" s="12"/>
     </row>
-    <row r="57" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
         <f t="shared" si="1"/>
         <v>56</v>
@@ -3881,7 +3881,7 @@
       <c r="P61" s="11"/>
       <c r="Q61" s="12"/>
     </row>
-    <row r="62" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
         <f t="shared" si="1"/>
         <v>61</v>
@@ -3923,7 +3923,7 @@
       <c r="P62" s="11"/>
       <c r="Q62" s="12"/>
     </row>
-    <row r="63" spans="1:17" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" s="13" customFormat="1" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5">
         <f t="shared" si="1"/>
         <v>62</v>
@@ -3965,7 +3965,7 @@
       <c r="P63" s="11"/>
       <c r="Q63" s="12"/>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5">
         <f t="shared" si="1"/>
         <v>63</v>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="L65" s="9"/>
     </row>
-    <row r="66" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="55">
         <f t="shared" si="1"/>
         <v>65</v>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="L68" s="24"/>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="46">
         <f t="shared" si="2"/>
         <v>68</v>
@@ -4185,7 +4185,7 @@
       </c>
       <c r="L69" s="9"/>
     </row>
-    <row r="70" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:12" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5">
         <f t="shared" si="2"/>
         <v>69</v>
@@ -4256,8 +4256,8 @@
       <c r="J71" s="18">
         <v>10000</v>
       </c>
-      <c r="K71" s="36">
-        <v>0</v>
+      <c r="K71" s="18">
+        <v>10000</v>
       </c>
       <c r="L71" s="9"/>
     </row>
@@ -4362,7 +4362,7 @@
       </c>
       <c r="L74" s="9"/>
     </row>
-    <row r="75" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:12" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5">
         <f t="shared" si="2"/>
         <v>74</v>
@@ -4399,7 +4399,7 @@
       </c>
       <c r="L75" s="9"/>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5">
         <f t="shared" si="2"/>
         <v>75</v>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="L82" s="42"/>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5">
         <f t="shared" si="2"/>
         <v>82</v>
@@ -4696,7 +4696,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5">
         <f t="shared" si="2"/>
         <v>84</v>
@@ -4772,7 +4772,7 @@
       </c>
       <c r="L86" s="9"/>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5">
         <f t="shared" si="2"/>
         <v>86</v>
@@ -4885,7 +4885,7 @@
       </c>
       <c r="L89" s="9"/>
     </row>
-    <row r="90" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:12" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5">
         <f t="shared" si="2"/>
         <v>89</v>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="L92" s="24"/>
     </row>
-    <row r="93" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:12" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5">
         <f t="shared" si="2"/>
         <v>92</v>
@@ -5173,7 +5173,7 @@
       </c>
       <c r="L97" s="9"/>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5">
         <f t="shared" si="2"/>
         <v>97</v>
@@ -5206,7 +5206,7 @@
       </c>
       <c r="L98" s="9"/>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:12" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5">
         <f t="shared" si="2"/>
         <v>98</v>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="K103" s="32">
         <f>COUNTIFS(E2:E98, "House", K2:K98, "&lt;&gt;0")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="104" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
@@ -5304,7 +5304,7 @@
       </c>
       <c r="K104" s="32">
         <f>COUNTIFS(E2:E98, "Apartment", K2:K98, "&lt;&gt;0")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="105" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="K105" s="32">
         <f>COUNTIFS(E2:E98, "Ind. Apartment", K2:K98, "&lt;&gt;0")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="106" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="K110" s="32">
         <f>COUNTIFS(D2:D98, "1st Main", K2:K98, "&lt;&gt;0")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="111" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="K111" s="32">
         <f>COUNTIFS(D2:D98, "2nd Main", K2:K98, "&lt;&gt;0")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="K112" s="32">
         <f>COUNTIFS(D2:D98, "3rd Main", K2:K98, "&lt;&gt;0")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="113" spans="5:11" ht="18.75" x14ac:dyDescent="0.3">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="K113" s="32">
         <f>COUNTIFS(D2:D98, "1st Cross", K2:K98, "&lt;&gt;0")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="114" spans="5:11" ht="18.75" x14ac:dyDescent="0.3">
@@ -5586,11 +5586,16 @@
       </c>
       <c r="K117" s="32">
         <f>COUNTIFS(D2:D98, "Seethammal Road", K2:K98, "&lt;&gt;0")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L98">
+  <autoFilter ref="A1:L99">
+    <filterColumn colId="10">
+      <filters>
+        <filter val="0.00"/>
+      </filters>
+    </filterColumn>
     <sortState ref="A2:J96">
       <sortCondition ref="D1:D96"/>
     </sortState>

</xml_diff>